<commit_message>
support temperature and humidity calibration workflows
</commit_message>
<xml_diff>
--- a/HM_19MB_Core/Resources/Templates/Tu_nhiet_3Pos.xlsx
+++ b/HM_19MB_Core/Resources/Templates/Tu_nhiet_3Pos.xlsx
@@ -5,16 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\Demo_HM_19MB\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\Demo_HM_19MB\HM_19MB_Demo\HM_19MB_Demo\Resources\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E492EC91-DC14-4C29-A873-D199EC53EF83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B6B4977-FE53-4132-8FFA-1E8DE4F2DF30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="3 Pos" sheetId="8" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'3 Pos'!$A$1:$AA$72</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="57">
   <si>
     <t>Cơ sở sản xuất:</t>
   </si>
@@ -377,6 +380,24 @@
       </rPr>
       <t>C</t>
     </r>
+  </si>
+  <si>
+    <t>Giá trị chuẩn, %RH</t>
+  </si>
+  <si>
+    <t>Điểm kiểm tra/ giá trị chỉ thị, %RH</t>
+  </si>
+  <si>
+    <t>Điểm kiểm tra/ Giá trị chỉ thị, %RH</t>
+  </si>
+  <si>
+    <t>Độ ổn định, %RH</t>
+  </si>
+  <si>
+    <t>Độ đồng đều, %RH</t>
+  </si>
+  <si>
+    <t>Độ không đảm bảo đo U (k=2, P=95%), %RH</t>
   </si>
 </sst>
 </file>
@@ -547,7 +568,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -594,12 +615,57 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -621,41 +687,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1102,7 +1135,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AA39"/>
+  <dimension ref="A1:AA40"/>
   <sheetFormatPr defaultColWidth="2.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.88671875" customWidth="1"/>
@@ -1133,43 +1166,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="50.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="28" t="s">
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="30" t="s">
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="30"/>
-      <c r="L1" s="30"/>
-      <c r="M1" s="30"/>
-      <c r="N1" s="30"/>
-      <c r="O1" s="36" t="s">
+      <c r="K1" s="45"/>
+      <c r="L1" s="45"/>
+      <c r="M1" s="45"/>
+      <c r="N1" s="45"/>
+      <c r="O1" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="P1" s="36"/>
-      <c r="Q1" s="36"/>
-      <c r="R1" s="36"/>
-      <c r="S1" s="36"/>
-      <c r="T1" s="36"/>
-      <c r="U1" s="43" t="s">
+      <c r="P1" s="46"/>
+      <c r="Q1" s="46"/>
+      <c r="R1" s="46"/>
+      <c r="S1" s="46"/>
+      <c r="T1" s="46"/>
+      <c r="U1" s="47" t="s">
         <v>38</v>
       </c>
-      <c r="V1" s="43"/>
-      <c r="W1" s="43"/>
-      <c r="X1" s="43"/>
-      <c r="Y1" s="43"/>
-      <c r="Z1" s="43"/>
-      <c r="AA1" s="43"/>
+      <c r="V1" s="47"/>
+      <c r="W1" s="47"/>
+      <c r="X1" s="47"/>
+      <c r="Y1" s="47"/>
+      <c r="Z1" s="47"/>
+      <c r="AA1" s="47"/>
     </row>
     <row r="2" spans="1:27" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7"/>
@@ -1183,17 +1216,17 @@
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
-      <c r="J2" s="33" t="s">
+      <c r="J2" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="K2" s="31" t="s">
+      <c r="K2" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="L2" s="32" t="s">
+      <c r="L2" s="33" t="s">
         <v>31</v>
       </c>
-      <c r="M2" s="32"/>
-      <c r="N2" s="32"/>
+      <c r="M2" s="33"/>
+      <c r="N2" s="33"/>
       <c r="Y2" t="s">
         <v>46</v>
       </c>
@@ -1213,8 +1246,8 @@
       <c r="G3" s="7"/>
       <c r="H3" s="7"/>
       <c r="I3" s="7"/>
-      <c r="J3" s="33"/>
-      <c r="K3" s="31"/>
+      <c r="J3" s="31"/>
+      <c r="K3" s="32"/>
       <c r="L3" s="21" t="s">
         <v>33</v>
       </c>
@@ -1224,67 +1257,67 @@
       <c r="N3" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="O3" s="39" t="s">
+      <c r="O3" s="34" t="s">
         <v>32</v>
       </c>
-      <c r="P3" s="34" t="s">
+      <c r="P3" s="36" t="s">
         <v>47</v>
       </c>
-      <c r="Q3" s="34" t="s">
+      <c r="Q3" s="36" t="s">
         <v>31</v>
       </c>
-      <c r="R3" s="34" t="s">
+      <c r="R3" s="36" t="s">
         <v>49</v>
       </c>
-      <c r="S3" s="34" t="s">
+      <c r="S3" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="T3" s="34" t="s">
+      <c r="T3" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="U3" s="37" t="s">
+      <c r="U3" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="V3" s="37" t="s">
+      <c r="V3" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="W3" s="37" t="s">
+      <c r="W3" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="X3" s="37" t="s">
+      <c r="X3" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="Y3" s="37" t="s">
+      <c r="Y3" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="Z3" s="41" t="s">
+      <c r="Z3" s="27" t="s">
         <v>45</v>
       </c>
-      <c r="AA3" s="37" t="s">
+      <c r="AA3" s="25" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:27" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="O4" s="40"/>
-      <c r="P4" s="35"/>
-      <c r="Q4" s="35"/>
-      <c r="R4" s="35"/>
-      <c r="S4" s="35"/>
-      <c r="T4" s="35"/>
-      <c r="U4" s="38"/>
-      <c r="V4" s="38"/>
-      <c r="W4" s="38"/>
-      <c r="X4" s="38"/>
-      <c r="Y4" s="38"/>
-      <c r="Z4" s="42"/>
-      <c r="AA4" s="38"/>
+      <c r="O4" s="35"/>
+      <c r="P4" s="37"/>
+      <c r="Q4" s="37"/>
+      <c r="R4" s="37"/>
+      <c r="S4" s="37"/>
+      <c r="T4" s="37"/>
+      <c r="U4" s="26"/>
+      <c r="V4" s="26"/>
+      <c r="W4" s="26"/>
+      <c r="X4" s="26"/>
+      <c r="Y4" s="26"/>
+      <c r="Z4" s="28"/>
+      <c r="AA4" s="26"/>
     </row>
     <row r="5" spans="1:27" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="6" spans="1:27" ht="22.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="38" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="22"/>
+      <c r="B6" s="38"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -1305,14 +1338,14 @@
       <c r="G7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H7" s="29"/>
-      <c r="I7" s="29"/>
+      <c r="H7" s="44"/>
+      <c r="I7" s="44"/>
     </row>
     <row r="8" spans="1:27" ht="22.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="22"/>
+      <c r="B8" s="38"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
@@ -1324,10 +1357,10 @@
       <c r="I8" s="2"/>
     </row>
     <row r="9" spans="1:27" ht="22.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="22"/>
+      <c r="B9" s="38"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
@@ -1337,12 +1370,12 @@
       <c r="I9" s="2"/>
     </row>
     <row r="10" spans="1:27" ht="22.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="25" t="s">
+      <c r="A10" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="25"/>
-      <c r="C10" s="26"/>
-      <c r="D10" s="26"/>
+      <c r="B10" s="40"/>
+      <c r="C10" s="41"/>
+      <c r="D10" s="41"/>
       <c r="E10" s="2" t="s">
         <v>23</v>
       </c>
@@ -1352,10 +1385,10 @@
       <c r="I10" s="2"/>
     </row>
     <row r="11" spans="1:27" ht="22.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="25"/>
+      <c r="B11" s="40"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2" t="s">
         <v>23</v>
@@ -1379,10 +1412,10 @@
       <c r="I12" s="2"/>
     </row>
     <row r="13" spans="1:27" ht="22.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="22" t="s">
+      <c r="A13" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="B13" s="22"/>
+      <c r="B13" s="38"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
@@ -1448,9 +1481,9 @@
       <c r="I17" s="2"/>
     </row>
     <row r="18" spans="1:9" ht="22.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="24"/>
-      <c r="B18" s="24"/>
-      <c r="C18" s="24"/>
+      <c r="A18" s="39"/>
+      <c r="B18" s="39"/>
+      <c r="C18" s="39"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
@@ -1634,7 +1667,7 @@
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
     </row>
-    <row r="33" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:27" ht="18" x14ac:dyDescent="0.35">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -1645,7 +1678,7 @@
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
     </row>
-    <row r="34" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:27" ht="18" x14ac:dyDescent="0.35">
       <c r="A34" s="23"/>
       <c r="B34" s="23"/>
       <c r="C34" s="23"/>
@@ -1656,7 +1689,7 @@
       <c r="H34" s="23"/>
       <c r="I34" s="23"/>
     </row>
-    <row r="36" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:27" ht="18" x14ac:dyDescent="0.35">
       <c r="A36" s="5"/>
       <c r="B36" s="5"/>
       <c r="C36" s="5"/>
@@ -1667,7 +1700,7 @@
       <c r="H36" s="5"/>
       <c r="I36" s="5"/>
     </row>
-    <row r="37" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:27" ht="36.6" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="5"/>
       <c r="B37" s="5"/>
       <c r="C37" s="5"/>
@@ -1677,8 +1710,32 @@
       <c r="G37" s="5"/>
       <c r="H37" s="5"/>
       <c r="I37" s="5"/>
-    </row>
-    <row r="38" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+      <c r="J37" s="29" t="s">
+        <v>9</v>
+      </c>
+      <c r="K37" s="30"/>
+      <c r="L37" s="30"/>
+      <c r="M37" s="30"/>
+      <c r="N37" s="30"/>
+      <c r="O37" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="P37" s="24"/>
+      <c r="Q37" s="24"/>
+      <c r="R37" s="24"/>
+      <c r="S37" s="24"/>
+      <c r="T37" s="24"/>
+      <c r="U37" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="V37" s="24"/>
+      <c r="W37" s="24"/>
+      <c r="X37" s="24"/>
+      <c r="Y37" s="24"/>
+      <c r="Z37" s="24"/>
+      <c r="AA37" s="24"/>
+    </row>
+    <row r="38" spans="1:27" ht="18" x14ac:dyDescent="0.35">
       <c r="A38" s="5"/>
       <c r="B38" s="5"/>
       <c r="C38" s="5"/>
@@ -1688,8 +1745,25 @@
       <c r="G38" s="5"/>
       <c r="H38" s="5"/>
       <c r="I38" s="5"/>
-    </row>
-    <row r="39" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+      <c r="J38" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="K38" s="32" t="s">
+        <v>52</v>
+      </c>
+      <c r="L38" s="33" t="s">
+        <v>51</v>
+      </c>
+      <c r="M38" s="33"/>
+      <c r="N38" s="33"/>
+      <c r="Y38" t="s">
+        <v>46</v>
+      </c>
+      <c r="Z38">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:27" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="5"/>
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
@@ -1699,9 +1773,74 @@
       <c r="G39" s="5"/>
       <c r="H39" s="5"/>
       <c r="I39" s="5"/>
+      <c r="J39" s="31"/>
+      <c r="K39" s="32"/>
+      <c r="L39" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="M39" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="N39" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="O39" s="34" t="s">
+        <v>32</v>
+      </c>
+      <c r="P39" s="36" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q39" s="36" t="s">
+        <v>51</v>
+      </c>
+      <c r="R39" s="36" t="s">
+        <v>54</v>
+      </c>
+      <c r="S39" s="36" t="s">
+        <v>55</v>
+      </c>
+      <c r="T39" s="36" t="s">
+        <v>56</v>
+      </c>
+      <c r="U39" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="V39" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="W39" s="25" t="s">
+        <v>41</v>
+      </c>
+      <c r="X39" s="25" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y39" s="25" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z39" s="27" t="s">
+        <v>45</v>
+      </c>
+      <c r="AA39" s="25" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="40" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="O40" s="35"/>
+      <c r="P40" s="37"/>
+      <c r="Q40" s="37"/>
+      <c r="R40" s="37"/>
+      <c r="S40" s="37"/>
+      <c r="T40" s="37"/>
+      <c r="U40" s="26"/>
+      <c r="V40" s="26"/>
+      <c r="W40" s="26"/>
+      <c r="X40" s="26"/>
+      <c r="Y40" s="26"/>
+      <c r="Z40" s="28"/>
+      <c r="AA40" s="26"/>
     </row>
   </sheetData>
-  <mergeCells count="34">
+  <mergeCells count="53">
     <mergeCell ref="X3:X4"/>
     <mergeCell ref="Y3:Y4"/>
     <mergeCell ref="Z3:Z4"/>
@@ -1736,6 +1875,25 @@
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A13:B13"/>
+    <mergeCell ref="J37:N37"/>
+    <mergeCell ref="J38:J39"/>
+    <mergeCell ref="K38:K39"/>
+    <mergeCell ref="L38:N38"/>
+    <mergeCell ref="O37:T37"/>
+    <mergeCell ref="O39:O40"/>
+    <mergeCell ref="P39:P40"/>
+    <mergeCell ref="Q39:Q40"/>
+    <mergeCell ref="R39:R40"/>
+    <mergeCell ref="S39:S40"/>
+    <mergeCell ref="T39:T40"/>
+    <mergeCell ref="U37:AA37"/>
+    <mergeCell ref="U39:U40"/>
+    <mergeCell ref="V39:V40"/>
+    <mergeCell ref="W39:W40"/>
+    <mergeCell ref="X39:X40"/>
+    <mergeCell ref="Y39:Y40"/>
+    <mergeCell ref="Z39:Z40"/>
+    <mergeCell ref="AA39:AA40"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>